<commit_message>
add code optimizations to refine_code parameter. add code diff and update readme.md file for code refinement changes. update Indicators.xlsx to correct data.
</commit_message>
<xml_diff>
--- a/Data point Supporting files/Germany 2017 (new)/Indicators.xlsx
+++ b/Data point Supporting files/Germany 2017 (new)/Indicators.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Indicators by country" sheetId="1" state="visible" r:id="rId2"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="346">
   <si>
     <t xml:space="preserve">Country</t>
   </si>
@@ -1061,6 +1061,9 @@
   </si>
   <si>
     <t xml:space="preserve">-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Disaster coping capacity</t>
   </si>
 </sst>
 </file>
@@ -1223,7 +1226,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Z1000"/>
-  <sheetFormatPr defaultColWidth="11.23828125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.2421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10.44"/>
@@ -10993,7 +10996,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F1000"/>
-  <sheetFormatPr defaultColWidth="11.23828125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.2421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.33"/>
@@ -12703,7 +12706,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B1000"/>
-  <sheetFormatPr defaultColWidth="11.23828125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.2421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="1" style="0" width="10.67"/>
   </cols>
@@ -13760,7 +13763,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C1000"/>
-  <sheetFormatPr defaultColWidth="11.23828125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.2421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="1" style="0" width="10.67"/>
   </cols>
@@ -15152,7 +15155,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:BU1000"/>
-  <sheetFormatPr defaultColWidth="11.23828125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.2421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="73" min="1" style="0" width="10.67"/>
   </cols>
@@ -24079,7 +24082,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F1000"/>
-  <sheetFormatPr defaultColWidth="11.23828125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.2421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="12" width="40.78"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="2" style="0" width="10.67"/>
@@ -25574,7 +25577,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C1000"/>
-  <sheetFormatPr defaultColWidth="11.23828125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.2421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="1" style="0" width="10.67"/>
   </cols>
@@ -25690,7 +25693,14 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="s">
+        <v>345</v>
+      </c>
+      <c r="C12" s="0" t="n">
+        <v>3</v>
+      </c>
+    </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>